<commit_message>
Updated board with new USB and changed 40 pin connector location. Need to reconnect leads on PCB Editor
</commit_message>
<xml_diff>
--- a/MechFighters_Badge_BOM_PCBWay.xlsx
+++ b/MechFighters_Badge_BOM_PCBWay.xlsx
@@ -152,7 +152,7 @@
     <t xml:space="preserve">SMD</t>
   </si>
   <si>
-    <t xml:space="preserve">D2, D3, D4, D5, D6, D7, D8</t>
+    <t xml:space="preserve">D2</t>
   </si>
   <si>
     <t xml:space="preserve">Lite-On Inc.</t>
@@ -589,76 +589,56 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -750,9 +730,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>666360</xdr:colOff>
+      <xdr:colOff>666000</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>156600</xdr:rowOff>
+      <xdr:rowOff>156240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -766,7 +746,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="209520"/>
-          <a:ext cx="1377000" cy="375840"/>
+          <a:ext cx="1376640" cy="375480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -878,32 +858,32 @@
       </c>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" s="14" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="8" t="s">
         <v>20</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="13"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
@@ -915,16 +895,16 @@
       <c r="C9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="8" t="s">
         <v>20</v>
       </c>
       <c r="H9" s="9" t="s">
@@ -1005,7 +985,7 @@
       <c r="F12" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G12" s="15"/>
+      <c r="G12" s="11"/>
       <c r="H12" s="9" t="s">
         <v>15</v>
       </c>
@@ -1021,7 +1001,7 @@
       <c r="C13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="12" t="s">
         <v>39</v>
       </c>
       <c r="E13" s="7" t="s">
@@ -1030,7 +1010,7 @@
       <c r="F13" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="15"/>
+      <c r="G13" s="11"/>
       <c r="H13" s="9" t="s">
         <v>15</v>
       </c>
@@ -1040,22 +1020,22 @@
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="F14" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="0" t="s">
+      <c r="G14" s="12" t="s">
         <v>46</v>
       </c>
       <c r="H14" s="9" t="s">
@@ -1073,7 +1053,7 @@
       <c r="C15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="12" t="s">
         <v>30</v>
       </c>
       <c r="E15" s="7" t="s">
@@ -1082,7 +1062,7 @@
       <c r="F15" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="11" t="s">
         <v>50</v>
       </c>
       <c r="H15" s="9" t="s">
@@ -1090,32 +1070,32 @@
       </c>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" s="14" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="16" t="s">
+      <c r="G16" s="11" t="s">
         <v>55</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="13"/>
+      <c r="I16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="n">
@@ -1136,7 +1116,7 @@
       <c r="F17" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G17" s="15" t="s">
+      <c r="G17" s="11" t="s">
         <v>60</v>
       </c>
       <c r="H17" s="9" t="s">
@@ -1154,7 +1134,7 @@
       <c r="C18" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="12" t="s">
         <v>30</v>
       </c>
       <c r="E18" s="7" t="s">
@@ -1163,7 +1143,7 @@
       <c r="F18" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="G18" s="11" t="s">
         <v>64</v>
       </c>
       <c r="H18" s="9" t="s">
@@ -1190,7 +1170,7 @@
       <c r="F19" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="15" t="s">
+      <c r="G19" s="11" t="s">
         <v>69</v>
       </c>
       <c r="H19" s="9" t="s">
@@ -1217,7 +1197,7 @@
       <c r="F20" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="G20" s="11" t="s">
         <v>74</v>
       </c>
       <c r="H20" s="9" t="s">
@@ -1229,22 +1209,22 @@
       <c r="A21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="12" t="s">
         <v>75</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="F21" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G21" s="0" t="s">
+      <c r="G21" s="12" t="s">
         <v>46</v>
       </c>
       <c r="H21" s="9" t="s">
@@ -1262,16 +1242,16 @@
       <c r="C22" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="E22" s="12" t="s">
         <v>78</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H22" s="9" t="s">
@@ -1282,22 +1262,22 @@
       <c r="A23" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="11" t="s">
+      <c r="C23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G23" s="16" t="s">
+      <c r="G23" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H23" s="9" t="s">
@@ -1308,49 +1288,49 @@
       <c r="A24" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="G24" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I24" s="18"/>
+      <c r="I24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="C25" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="G25" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H25" s="9" t="s">
@@ -1364,7 +1344,7 @@
       <c r="B26" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C26" s="10" t="n">
+      <c r="C26" s="6" t="n">
         <v>27</v>
       </c>
       <c r="D26" s="1" t="s">
@@ -1376,7 +1356,7 @@
       <c r="F26" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G26" s="16" t="s">
+      <c r="G26" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H26" s="9" t="s">
@@ -1390,10 +1370,10 @@
       <c r="B27" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C27" s="10" t="n">
+      <c r="C27" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="7" t="s">
         <v>82</v>
       </c>
       <c r="E27" s="1" t="s">
@@ -1402,7 +1382,7 @@
       <c r="F27" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H27" s="9" t="s">
@@ -1416,7 +1396,7 @@
       <c r="B28" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C28" s="10" t="n">
+      <c r="C28" s="6" t="n">
         <v>8</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -1428,7 +1408,7 @@
       <c r="F28" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="G28" s="16" t="s">
+      <c r="G28" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H28" s="9" t="s">
@@ -1439,22 +1419,22 @@
       <c r="A29" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C29" s="10" t="n">
+      <c r="C29" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D29" s="0" t="s">
+      <c r="D29" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="E29" s="0" t="s">
+      <c r="E29" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="F29" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="G29" s="16" t="s">
+      <c r="G29" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H29" s="9" t="s">
@@ -1465,22 +1445,22 @@
       <c r="A30" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C30" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="0" t="s">
+      <c r="C30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="E30" s="0" t="s">
+      <c r="E30" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="F30" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="G30" s="16" t="s">
+      <c r="G30" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H30" s="9" t="s">
@@ -1502,14 +1482,14 @@
       <c r="F31" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="G31" s="16"/>
+      <c r="G31" s="11"/>
       <c r="H31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="12" t="s">
         <v>112</v>
       </c>
       <c r="C32" s="6" t="n">
@@ -1525,7 +1505,7 @@
       <c r="A33" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="12" t="s">
         <v>113</v>
       </c>
       <c r="C33" s="6" t="n">
@@ -1541,7 +1521,7 @@
       <c r="A34" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="12" t="s">
         <v>114</v>
       </c>
       <c r="C34" s="6" t="n">
@@ -1554,23 +1534,23 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0"/>
-      <c r="B35" s="0"/>
-      <c r="C35" s="0" t="n">
+      <c r="A35" s="12"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="12" t="n">
         <f aca="false">SUM(C7:C34)</f>
         <v>84</v>
       </c>
-      <c r="D35" s="0"/>
-      <c r="E35" s="0"/>
-      <c r="F35" s="0"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0"/>
-      <c r="B36" s="0"/>
-      <c r="C36" s="0"/>
-      <c r="D36" s="0"/>
-      <c r="E36" s="0"/>
-      <c r="F36" s="0"/>
+      <c r="A36" s="12"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1598,7 +1578,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="17" width="9"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="12" width="9"/>
   </cols>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1619,7 +1599,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="17" width="9"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="12" width="9"/>
   </cols>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Flipped LED positions, names, added back display silksaw.
</commit_message>
<xml_diff>
--- a/MechFighters_Badge_BOM_PCBWay.xlsx
+++ b/MechFighters_Badge_BOM_PCBWay.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="115">
   <si>
     <t xml:space="preserve">CPEC Mechfighters Badge Rev 1, 84PCS BOM  (Bill of Materials)</t>
   </si>
@@ -209,10 +209,10 @@
     <t xml:space="preserve">J1</t>
   </si>
   <si>
-    <t xml:space="preserve">Hirose Electric Co Ltd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CX90B-16P1</t>
+    <t xml:space="preserve">Same Sky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UJ20-C-H-G-SMT-5-P16-TR</t>
   </si>
   <si>
     <t xml:space="preserve">USB-C (USB TYPE-C)</t>
@@ -1493,13 +1493,11 @@
         <v>112</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
-      <c r="F32" s="7" t="s">
-        <v>111</v>
-      </c>
+      <c r="F32" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="n">
@@ -1538,7 +1536,7 @@
       <c r="B35" s="12"/>
       <c r="C35" s="12" t="n">
         <f aca="false">SUM(C7:C34)</f>
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="12"/>

</xml_diff>

<commit_message>
Updates to H-Bridge design.
</commit_message>
<xml_diff>
--- a/MechFighters_Badge_BOM_PCBWay.xlsx
+++ b/MechFighters_Badge_BOM_PCBWay.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="112">
   <si>
     <t xml:space="preserve">CPEC Mechfighters Badge Rev 1, 84PCS BOM  (Bill of Materials)</t>
   </si>
@@ -152,30 +152,21 @@
     <t xml:space="preserve">SMD</t>
   </si>
   <si>
-    <t xml:space="preserve">D2</t>
+    <t xml:space="preserve">D9, D10, D11, D12, D13, D14</t>
   </si>
   <si>
     <t xml:space="preserve">Lite-On Inc.</t>
   </si>
   <si>
-    <t xml:space="preserve">LTST-C190KSKT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LED YELLOW CLEAR CHIP SMD</t>
+    <t xml:space="preserve">LTST-C190KRKT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED RED CLEAR CHIP SMD</t>
   </si>
   <si>
     <t xml:space="preserve">0603 (1608 Metric)</t>
   </si>
   <si>
-    <t xml:space="preserve">D9, D10, D11, D12, D13, D14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LTST-C190KRKT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LED RED CLEAR CHIP SMD</t>
-  </si>
-  <si>
     <t xml:space="preserve">Q1</t>
   </si>
   <si>
@@ -368,7 +359,7 @@
     <t xml:space="preserve">100 k</t>
   </si>
   <si>
-    <t xml:space="preserve">R5, R6, R7, R8</t>
+    <t xml:space="preserve">R5, R6, R7</t>
   </si>
   <si>
     <t xml:space="preserve">Stackpole Electronics Inc</t>
@@ -437,7 +428,7 @@
     <t xml:space="preserve">J3, J4, J5, J6, J7</t>
   </si>
   <si>
-    <t xml:space="preserve">DNC (Do Not Connect)</t>
+    <t xml:space="preserve">DNP (Do not Populate)</t>
   </si>
   <si>
     <t xml:space="preserve">SW1, SW2, SW3, SW4, SW5, SW6, SW7, SW8, SW9, SW10, SW11, SW12</t>
@@ -730,9 +721,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>666000</xdr:colOff>
+      <xdr:colOff>665280</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>156240</xdr:rowOff>
+      <xdr:rowOff>155520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -746,7 +737,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="209520"/>
-          <a:ext cx="1376640" cy="375480"/>
+          <a:ext cx="1375920" cy="374760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -859,30 +850,14 @@
       <c r="I7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>15</v>
-      </c>
+      <c r="A8" s="6"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="9"/>
       <c r="I8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -890,7 +865,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>6</v>
@@ -899,10 +874,10 @@
         <v>17</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>20</v>
@@ -917,22 +892,22 @@
         <v>4</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>28</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>15</v>
@@ -944,22 +919,22 @@
         <v>5</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="G11" s="8" t="s">
         <v>30</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>33</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>15</v>
@@ -971,19 +946,19 @@
         <v>6</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>34</v>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>37</v>
       </c>
       <c r="G12" s="11"/>
       <c r="H12" s="9" t="s">
@@ -996,19 +971,19 @@
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="G13" s="11"/>
       <c r="H13" s="9" t="s">
@@ -1021,22 +996,22 @@
         <v>8</v>
       </c>
       <c r="B14" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="12" t="s">
+      <c r="G14" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>46</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>15</v>
@@ -1048,22 +1023,22 @@
         <v>9</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="11" t="s">
         <v>47</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>50</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>15</v>
@@ -1075,22 +1050,22 @@
         <v>10</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="G16" s="11" t="s">
         <v>52</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>55</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>15</v>
@@ -1102,22 +1077,22 @@
         <v>11</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="7" t="s">
+      <c r="G17" s="11" t="s">
         <v>57</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>60</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>15</v>
@@ -1129,22 +1104,22 @@
         <v>12</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="11" t="s">
         <v>61</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>64</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>15</v>
@@ -1156,22 +1131,22 @@
         <v>13</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F19" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="7" t="s">
+      <c r="G19" s="11" t="s">
         <v>66</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="H19" s="9" t="s">
         <v>15</v>
@@ -1183,22 +1158,22 @@
         <v>14</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="7" t="s">
+      <c r="G20" s="11" t="s">
         <v>71</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>74</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>15</v>
@@ -1210,22 +1185,22 @@
         <v>15</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G21" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>46</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>15</v>
@@ -1237,22 +1212,22 @@
         <v>16</v>
       </c>
       <c r="B22" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="12" t="s">
+      <c r="G22" s="11" t="s">
         <v>77</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>80</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>15</v>
@@ -1263,22 +1238,22 @@
         <v>17</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>84</v>
-      </c>
       <c r="G23" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H23" s="9" t="s">
         <v>15</v>
@@ -1289,22 +1264,22 @@
         <v>18</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>15</v>
@@ -1316,22 +1291,22 @@
         <v>19</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F25" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>91</v>
-      </c>
       <c r="G25" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>15</v>
@@ -1342,22 +1317,22 @@
         <v>20</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>27</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H26" s="9" t="s">
         <v>15</v>
@@ -1368,22 +1343,22 @@
         <v>21</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C27" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H27" s="9" t="s">
         <v>15</v>
@@ -1394,22 +1369,22 @@
         <v>22</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>8</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H28" s="9" t="s">
         <v>15</v>
@@ -1420,22 +1395,22 @@
         <v>23</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>12</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H29" s="9" t="s">
         <v>15</v>
@@ -1446,22 +1421,22 @@
         <v>24</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="F30" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="E30" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>109</v>
-      </c>
       <c r="G30" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H30" s="9" t="s">
         <v>15</v>
@@ -1472,7 +1447,7 @@
         <v>25</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>0</v>
@@ -1480,7 +1455,7 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G31" s="11"/>
       <c r="H31" s="9"/>
@@ -1490,21 +1465,23 @@
         <v>26</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
+      <c r="F32" s="7" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="n">
         <v>27</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>0</v>
@@ -1512,7 +1489,7 @@
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
       <c r="F33" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1520,7 +1497,7 @@
         <v>28</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C34" s="6" t="n">
         <v>0</v>
@@ -1528,7 +1505,7 @@
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
       <c r="F34" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1536,7 +1513,7 @@
       <c r="B35" s="12"/>
       <c r="C35" s="12" t="n">
         <f aca="false">SUM(C7:C34)</f>
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="12"/>

</xml_diff>

<commit_message>
Added sideview LED to BOM.
</commit_message>
<xml_diff>
--- a/MechFighters_Badge_BOM_PCBWay.xlsx
+++ b/MechFighters_Badge_BOM_PCBWay.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="115">
   <si>
     <t xml:space="preserve">CPEC Mechfighters Badge Rev 1, 84PCS BOM  (Bill of Materials)</t>
   </si>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">SMD</t>
   </si>
   <si>
-    <t xml:space="preserve">D9, D10, D11, D12, D13, D14</t>
+    <t xml:space="preserve">D3, D4, D5, D7, D8</t>
   </si>
   <si>
     <t xml:space="preserve">Lite-On Inc.</t>
@@ -438,6 +438,15 @@
   </si>
   <si>
     <t xml:space="preserve">R38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Würth Elektronik </t>
+  </si>
+  <si>
+    <t xml:space="preserve">155124YS73200</t>
   </si>
 </sst>
 </file>
@@ -721,9 +730,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>665280</xdr:colOff>
+      <xdr:colOff>664920</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>155520</xdr:rowOff>
+      <xdr:rowOff>155160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -737,7 +746,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="209520"/>
-          <a:ext cx="1375920" cy="374760"/>
+          <a:ext cx="1375560" cy="374400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1510,19 +1519,27 @@
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12" t="n">
-        <f aca="false">SUM(C7:C34)</f>
-        <v>78</v>
-      </c>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
+      <c r="B35" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>114</v>
+      </c>
       <c r="F35" s="12"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12"/>
       <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
+      <c r="C36" s="12" t="n">
+        <f aca="false">SUM(C7:C34)</f>
+        <v>78</v>
+      </c>
       <c r="D36" s="12"/>
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>

</xml_diff>

<commit_message>
Made adjustments to silkscreen, resolved a few more design rule check warnings.
</commit_message>
<xml_diff>
--- a/MechFighters_Badge_BOM_PCBWay.xlsx
+++ b/MechFighters_Badge_BOM_PCBWay.xlsx
@@ -22,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="115">
-  <si>
-    <t xml:space="preserve">CPEC Mechfighters Badge Rev 1, 84PCS BOM  (Bill of Materials)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="113">
+  <si>
+    <t xml:space="preserve">CPEC Mechfighters Badge Rev 2, 84PCS BOM  (Bill of Materials)</t>
   </si>
   <si>
     <t xml:space="preserve">Item #</t>
@@ -329,124 +329,118 @@
     <t xml:space="preserve">1210</t>
   </si>
   <si>
+    <t xml:space="preserve">R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic Electronic Components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERJ-2GEJ5R1X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1 ohms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YAGEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0402FR-071ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3, R4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0402FR-07100KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5, R6, R7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stackpole Electronics Inc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RMCF0402FT10K0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R9, R10, R11, R12, R13, R14, R15, R16, R17, R18, R19, R20, R21, R22, R23, R24, R25, R26, R27, R28, R29, R30, R32, R33, R34, R35, R36, R37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0402FR-075K1L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1 k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1, C2, C3, C4, C5, C6, C7, C8, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata Electronics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM155R61A106ME11D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C9, C10, C11, C12, C13, C14, C15, C16, C17, C18, C19, C20, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEMET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C0402C105K9PACTU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walsin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0402B104K160CT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1 uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J3, J4, J5, J6, J7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DNP (Do not Populate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THT</t>
+  </si>
+  <si>
     <t xml:space="preserve">SW1</t>
   </si>
   <si>
-    <t xml:space="preserve">R1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panasonic Electronic Components</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERJ-2GEJ5R1X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.1 ohms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YAGEO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RC0402FR-071ML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3, R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RC0402FR-07100KL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5, R6, R7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stackpole Electronics Inc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RMCF0402FT10K0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R9, R10, R11, R12, R13, R14, R15, R16, R17, R18, R19, R20, R21, R22, R23, R24, R25, R26, R27, R28, R29, R30, R32, R33, R34, R35, R36, R37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RC0402FR-075K1L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.1 k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1, C2, C3, C4, C5, C6, C7, C8, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Murata Electronics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRM155R61A106ME11D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C9, C10, C11, C12, C13, C14, C15, C16, C17, C18, C19, C20, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEMET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C0402C105K9PACTU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walsin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0402B104K160CT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1 uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J3, J4, J5, J6, J7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNP (Do not Populate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SW1, SW2, SW3, SW4, SW5, SW6, SW7, SW8, SW9, SW10, SW11, SW12</t>
+    <t xml:space="preserve">SW2, SW3, SW4, SW5, SW6, SW7, SW8, SW9, SW10, SW11, SW12</t>
   </si>
   <si>
     <t xml:space="preserve">BZ1</t>
   </si>
   <si>
     <t xml:space="preserve">R38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Würth Elektronik </t>
-  </si>
-  <si>
-    <t xml:space="preserve">155124YS73200</t>
   </si>
 </sst>
 </file>
@@ -634,12 +628,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -648,13 +642,13 @@
     </xf>
   </cellXfs>
   <cellStyles count="7">
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8" customBuiltin="false"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -730,9 +724,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>664560</xdr:colOff>
+      <xdr:colOff>664200</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>154800</xdr:rowOff>
+      <xdr:rowOff>154440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -745,13 +739,13 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9360" y="209160"/>
-          <a:ext cx="1274040" cy="374040"/>
+          <a:off x="9360" y="209520"/>
+          <a:ext cx="1364040" cy="373680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln w="0">
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
@@ -762,23 +756,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:I65536"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A2:I1048576"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" hidden="false" max="1" min="1" style="1" width="8.8659793814433"/>
-    <col collapsed="false" hidden="false" max="2" min="2" style="1" width="26.4587628865979"/>
-    <col collapsed="false" hidden="false" max="3" min="3" style="1" width="8.8659793814433"/>
-    <col collapsed="false" hidden="false" max="4" min="4" style="1" width="33.2783505154639"/>
-    <col collapsed="false" hidden="false" max="5" min="5" style="1" width="29.7319587628866"/>
-    <col collapsed="false" hidden="false" max="6" min="6" style="1" width="41.4587628865979"/>
-    <col collapsed="false" hidden="false" max="7" min="7" style="1" width="20.7319587628866"/>
-    <col collapsed="false" hidden="false" max="8" min="8" style="1" width="13.5"/>
-    <col collapsed="false" hidden="false" max="9" min="9" style="1" width="35.4587628865979"/>
-    <col collapsed="false" hidden="false" max="1025" min="10" style="1" width="8.8659793814433"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="33.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="29.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="41.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="35.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="10" style="1" width="8.86"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -922,10 +916,10 @@
       <c r="C10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="11" t="s">
         <v>26</v>
       </c>
       <c r="F10" s="8" t="s">
@@ -985,7 +979,7 @@
       <c r="F12" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G12" s="11"/>
+      <c r="G12" s="12"/>
       <c r="H12" s="9" t="s">
         <v>15</v>
       </c>
@@ -1001,7 +995,7 @@
       <c r="C13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="11" t="s">
         <v>39</v>
       </c>
       <c r="E13" s="7" t="s">
@@ -1010,7 +1004,7 @@
       <c r="F13" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="11"/>
+      <c r="G13" s="12"/>
       <c r="H13" s="9" t="s">
         <v>15</v>
       </c>
@@ -1020,22 +1014,22 @@
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>42</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="G14" s="11" t="s">
         <v>46</v>
       </c>
       <c r="H14" s="9" t="s">
@@ -1053,7 +1047,7 @@
       <c r="C15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="11" t="s">
         <v>30</v>
       </c>
       <c r="E15" s="7" t="s">
@@ -1062,7 +1056,7 @@
       <c r="F15" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="12" t="s">
         <v>50</v>
       </c>
       <c r="H15" s="9" t="s">
@@ -1089,7 +1083,7 @@
       <c r="F16" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="12" t="s">
         <v>55</v>
       </c>
       <c r="H16" s="9" t="s">
@@ -1116,7 +1110,7 @@
       <c r="F17" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="12" t="s">
         <v>60</v>
       </c>
       <c r="H17" s="9" t="s">
@@ -1134,7 +1128,7 @@
       <c r="C18" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="11" t="s">
         <v>30</v>
       </c>
       <c r="E18" s="7" t="s">
@@ -1143,7 +1137,7 @@
       <c r="F18" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="12" t="s">
         <v>64</v>
       </c>
       <c r="H18" s="9" t="s">
@@ -1170,7 +1164,7 @@
       <c r="F19" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="12" t="s">
         <v>69</v>
       </c>
       <c r="H19" s="9" t="s">
@@ -1197,7 +1191,7 @@
       <c r="F20" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="12" t="s">
         <v>74</v>
       </c>
       <c r="H20" s="9" t="s">
@@ -1207,25 +1201,25 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>75</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>45</v>
+      <c r="D21" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>78</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>15</v>
@@ -1234,25 +1228,25 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>78</v>
+      <c r="D22" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>82</v>
       </c>
       <c r="F22" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>79</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>80</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>15</v>
@@ -1260,25 +1254,25 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="E23" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G23" s="11" t="s">
-        <v>80</v>
+        <v>86</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>79</v>
       </c>
       <c r="H23" s="9" t="s">
         <v>15</v>
@@ -1286,25 +1280,25 @@
     </row>
     <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="G24" s="11" t="s">
-        <v>80</v>
+        <v>90</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>79</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>15</v>
@@ -1313,25 +1307,25 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>88</v>
+        <v>20</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G25" s="11" t="s">
-        <v>80</v>
+        <v>27</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>79</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>15</v>
@@ -1339,58 +1333,77 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G26" s="11" t="s">
-        <v>80</v>
+        <v>97</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>79</v>
       </c>
       <c r="H26" s="9" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="7"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="9"/>
+      <c r="A27" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>95</v>
+        <v>24</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>102</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>80</v>
+        <v>1</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>79</v>
       </c>
       <c r="H28" s="9" t="s">
         <v>15</v>
@@ -1398,62 +1411,50 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>99</v>
+        <v>25</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>106</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="E29" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="F29" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>80</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G29" s="12"/>
       <c r="H29" s="9" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>103</v>
+        <v>15</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>109</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="E30" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>80</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G30" s="11"/>
       <c r="H30" s="9" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>107</v>
+        <v>26</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>110</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>0</v>
@@ -1461,17 +1462,18 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>109</v>
+        <v>27</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>111</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>0</v>
@@ -1479,15 +1481,18 @@
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
       <c r="F32" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>110</v>
+        <v>28</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>112</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>0</v>
@@ -1495,51 +1500,40 @@
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
       <c r="F33" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="C34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7" t="s">
-        <v>108</v>
-      </c>
+      <c r="A34" s="0"/>
+      <c r="B34" s="0"/>
+      <c r="C34" s="0"/>
+      <c r="D34" s="0"/>
+      <c r="E34" s="0"/>
+      <c r="F34" s="0"/>
+      <c r="G34" s="0"/>
+      <c r="H34" s="0"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12"/>
-      <c r="B35" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C35" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F35" s="12"/>
+      <c r="A35" s="11"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12" t="n">
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11" t="n">
         <f aca="false">SUM(C7:C34)</f>
-        <v>76</v>
-      </c>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
+        <v>75</v>
+      </c>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1549,8 +1543,8 @@
     <mergeCell ref="D2:F4"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.699305555555555" right="0.699305555555555" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1560,19 +1554,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" hidden="false" max="1025" min="1" style="12" width="8.8659793814433"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="1" style="11" width="8.86"/>
   </cols>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.699305555555555" right="0.699305555555555" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1581,19 +1575,19 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" hidden="false" max="1025" min="1" style="12" width="8.8659793814433"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="1" style="11" width="8.86"/>
   </cols>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.699305555555555" right="0.699305555555555" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>